<commit_message>
slettet alle unødvendige kompileringsfiler
</commit_message>
<xml_diff>
--- a/TermProject/state_table.xlsx
+++ b/TermProject/state_table.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="109">
   <si>
     <t xml:space="preserve">Inputs</t>
   </si>
@@ -173,6 +173,18 @@
     <t xml:space="preserve">if counter &gt;= n</t>
   </si>
   <si>
+    <t xml:space="preserve">S5[256]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4[256]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3[256]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2[256]</t>
+  </si>
+  <si>
     <t xml:space="preserve">mux_ctrl_R_in[3..0]</t>
   </si>
   <si>
@@ -182,28 +194,22 @@
     <t xml:space="preserve">A[255]</t>
   </si>
   <si>
-    <t xml:space="preserve">R_sel[3..0]</t>
+    <t xml:space="preserve">R_sel[2..0]</t>
   </si>
   <si>
     <t xml:space="preserve">Boolean Function</t>
   </si>
   <si>
-    <t xml:space="preserve">S5[256]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S4[256]</t>
-  </si>
-  <si>
     <t xml:space="preserve">b101</t>
   </si>
   <si>
     <t xml:space="preserve">S5</t>
   </si>
   <si>
-    <t xml:space="preserve">nor(A, MR[3])</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S3[256]</t>
+    <t xml:space="preserve">and(A, not(MR[3]))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S5 = R  + b – 2*n</t>
   </si>
   <si>
     <t xml:space="preserve">S4</t>
@@ -215,7 +221,7 @@
     <t xml:space="preserve">and(A, MR[2])</t>
   </si>
   <si>
-    <t xml:space="preserve">S2[256]</t>
+    <t xml:space="preserve">S4 = R – 2*n</t>
   </si>
   <si>
     <t xml:space="preserve">S3</t>
@@ -227,6 +233,9 @@
     <t xml:space="preserve">nor(A, MR[3], MR[1])</t>
   </si>
   <si>
+    <t xml:space="preserve">S3 = R + b – n</t>
+  </si>
+  <si>
     <t xml:space="preserve">S2</t>
   </si>
   <si>
@@ -236,6 +245,9 @@
     <t xml:space="preserve">and(A, MR[2], MR[0])</t>
   </si>
   <si>
+    <t xml:space="preserve">S2 = R – n</t>
+  </si>
+  <si>
     <t xml:space="preserve">S1</t>
   </si>
   <si>
@@ -245,12 +257,18 @@
     <t xml:space="preserve">and(A, MR[3], MR[1])</t>
   </si>
   <si>
+    <t xml:space="preserve">S1 = R + b</t>
+  </si>
+  <si>
     <t xml:space="preserve">S0</t>
   </si>
   <si>
     <t xml:space="preserve">b000</t>
   </si>
   <si>
+    <t xml:space="preserve">S0 = R</t>
+  </si>
+  <si>
     <t xml:space="preserve">Forkortelser:</t>
   </si>
   <si>
@@ -261,6 +279,15 @@
   </si>
   <si>
     <t xml:space="preserve">mux_ctrl_R_in[]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R_sel[0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">R_sel[1]</t>
   </si>
   <si>
     <t xml:space="preserve">mux_ctrl_P_in[3..0]</t>
@@ -1598,31 +1625,43 @@
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
+      <c r="F15" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="K16" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="L16" s="7"/>
       <c r="M16" s="8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="N16" s="1"/>
     </row>
@@ -1631,7 +1670,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D17" s="8"/>
       <c r="F17" s="8" t="n">
@@ -1653,16 +1692,16 @@
         <v>2</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
@@ -1677,31 +1716,33 @@
         <v>0</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="N18" s="1"/>
+        <v>61</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>58</v>
-      </c>
       <c r="E19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>0</v>
@@ -1716,31 +1757,33 @@
         <v>1</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="N19" s="1"/>
+        <v>65</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>0</v>
@@ -1755,25 +1798,27 @@
         <v>0</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="N20" s="1"/>
+        <v>69</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C21" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0</v>
@@ -1788,25 +1833,27 @@
         <v>1</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="N21" s="1"/>
+        <v>73</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -1821,26 +1868,28 @@
         <v>0</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="N22" s="1"/>
+        <v>77</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1"/>
       <c r="C23" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -1855,25 +1904,27 @@
         <v>1</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="N23" s="1"/>
+        <v>73</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C24" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0</v>
@@ -1891,13 +1942,13 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0</v>
@@ -1916,13 +1967,13 @@
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8"/>
       <c r="C26" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>1</v>
@@ -1937,25 +1988,25 @@
         <v>0</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="N26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C27" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>1</v>
@@ -1971,22 +2022,22 @@
       </c>
       <c r="K27" s="1"/>
       <c r="L27" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="N27" s="1"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>1</v>
@@ -2007,13 +2058,13 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C29" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>1</v>
@@ -2032,13 +2083,13 @@
       <c r="A30" s="1"/>
       <c r="B30" s="10"/>
       <c r="C30" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>1</v>
@@ -2051,18 +2102,24 @@
       </c>
       <c r="I30" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1"/>
       <c r="C31" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>1</v>
@@ -2075,17 +2132,20 @@
       </c>
       <c r="I31" s="2" t="n">
         <v>1</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C32" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" s="2" t="n">
         <v>1</v>
@@ -2102,13 +2162,13 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>1</v>
@@ -2125,13 +2185,13 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
@@ -2148,13 +2208,13 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C35" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0</v>
@@ -2171,13 +2231,13 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C36" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
         <v>0</v>
@@ -2194,13 +2254,13 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C37" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0</v>
@@ -2217,13 +2277,13 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C38" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>0</v>
@@ -2240,13 +2300,13 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C39" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>0</v>
@@ -2263,13 +2323,13 @@
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C40" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>0</v>
@@ -2286,13 +2346,13 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C41" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
@@ -2309,13 +2369,13 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C42" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>1</v>
@@ -2332,13 +2392,13 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>1</v>
@@ -2355,13 +2415,13 @@
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>1</v>
@@ -2378,13 +2438,13 @@
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C45" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>1</v>
@@ -2401,13 +2461,13 @@
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C46" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
         <v>1</v>
@@ -2424,13 +2484,13 @@
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C47" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>1</v>
@@ -2447,13 +2507,13 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C48" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F48" s="2" t="n">
         <v>1</v>
@@ -2470,13 +2530,13 @@
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C49" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F49" s="2" t="n">
         <v>1</v>
@@ -2555,27 +2615,27 @@
     <row r="63" customFormat="false" ht="14.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D66" s="7"/>
       <c r="E66" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G66" s="7"/>
       <c r="H66" s="7"/>
       <c r="I66" s="7"/>
       <c r="K66" s="7" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="L66" s="7"/>
       <c r="M66" s="8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="N66" s="1"/>
     </row>
@@ -2584,7 +2644,7 @@
         <v>3</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F67" s="8" t="n">
         <v>3</v>
@@ -2605,13 +2665,13 @@
         <v>2</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>0</v>
@@ -2629,13 +2689,13 @@
         <v>0</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M68" s="5" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="N68" s="1"/>
     </row>
@@ -2644,13 +2704,13 @@
         <v>1</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>0</v>
@@ -2668,13 +2728,13 @@
         <v>1</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M69" s="5" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="N69" s="1"/>
     </row>
@@ -2683,13 +2743,13 @@
         <v>0</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>0</v>
@@ -2707,22 +2767,22 @@
         <v>0</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="N70" s="1"/>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C71" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>0</v>
@@ -2740,22 +2800,22 @@
         <v>1</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="N71" s="1"/>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C72" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>0</v>
@@ -2773,22 +2833,22 @@
         <v>0</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="N72" s="1"/>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C73" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>0</v>
@@ -2806,22 +2866,22 @@
         <v>1</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="M73" s="5" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="N73" s="1"/>
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C74" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>0</v>
@@ -2842,10 +2902,10 @@
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C75" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>0</v>
@@ -2866,10 +2926,10 @@
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C76" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>0</v>
@@ -2887,22 +2947,22 @@
         <v>0</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="L76" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="N76" s="1"/>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C77" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>0</v>
@@ -2921,19 +2981,19 @@
       </c>
       <c r="K77" s="1"/>
       <c r="L77" s="5" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="M77" s="5" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="N77" s="1"/>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C78" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>0</v>
@@ -2953,10 +3013,10 @@
     </row>
     <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C79" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>0</v>
@@ -2976,10 +3036,10 @@
     </row>
     <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C80" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>0</v>
@@ -2999,10 +3059,10 @@
     </row>
     <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C81" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>0</v>
@@ -3022,10 +3082,10 @@
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C82" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>0</v>
@@ -3045,10 +3105,10 @@
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C83" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>0</v>
@@ -3068,10 +3128,10 @@
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C84" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>1</v>
@@ -3091,10 +3151,10 @@
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C85" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>1</v>
@@ -3114,10 +3174,10 @@
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C86" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>1</v>
@@ -3137,10 +3197,10 @@
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C87" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>1</v>
@@ -3160,10 +3220,10 @@
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C88" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>1</v>
@@ -3183,10 +3243,10 @@
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C89" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>1</v>
@@ -3206,10 +3266,10 @@
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C90" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D90" s="8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>1</v>
@@ -3229,10 +3289,10 @@
     </row>
     <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C91" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>1</v>
@@ -3252,10 +3312,10 @@
     </row>
     <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C92" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>1</v>
@@ -3275,10 +3335,10 @@
     </row>
     <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C93" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>1</v>
@@ -3298,10 +3358,10 @@
     </row>
     <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C94" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D94" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>1</v>
@@ -3321,10 +3381,10 @@
     </row>
     <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C95" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>1</v>
@@ -3344,10 +3404,10 @@
     </row>
     <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C96" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>1</v>
@@ -3367,10 +3427,10 @@
     </row>
     <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C97" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D97" s="8" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>1</v>
@@ -3390,10 +3450,10 @@
     </row>
     <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C98" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D98" s="8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>1</v>
@@ -3413,10 +3473,10 @@
     </row>
     <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C99" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D99" s="8" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>1</v>

</xml_diff>